<commit_message>
[36차] Stage2Group 대사/연출 보정 + CodexGroup 기본 틀 + BGM 전환 + HUD/Dialogue 개선 + 스키마 수정 및 최신화
이번 커밋은 Stage2Group 2차 작업과 함께, 프로젝트 전체 구조를 대대적으로 개편하고 스키마를 수정 및 최신화한 커밋입니다.

주요 변경 내용:

- Stage2Group 2차 작업 진행 (대사 흐름, 연출, NPC 배치 등 보완)

- 전체 구조 대대적 개편
  - 참조 중심 구조 → 컴포넌트 기반 + 데이터/매니저 드리븐 중심으로 전환
  - Controller가 너무 많은 오브젝트를 직접 참조하던 방식 개선
  - 각 오브젝트(배우)에 자기 역할 컴포넌트를 붙이는 구조로 변경
  - 느슨한 결합과 재사용성 대폭 향상

- 스키마 수정 및 최신화
  - OO_Stage, OO_StageQuest, OO_Ingredient 등 스키마 정리 및 업데이트
  - JSON Output 재생성 및 데이터 드리븐 안정화

- BGM 업데이트 및 전환 로직 보강
  - Stage2 진입 시 적절한 BGM으로 전환
  - Road → Stage 간 BGM 연속성 개선

이번 개편의 목적:
강사님 피드백(참조보단 컴포넌트)을 보다 철저히 반영하고,
나중에 팀 작업을 할 때도 다른 사람이 쉽게 이해하고 확장할 수 있는 구조로 만들기 위함입니다.

현재 Make it Work 상태:
- Stage2Group 2차 작업 완료
- 전체 구조가 이전보다 훨씬 깔끔하고 확장하기 쉬워짐
- 데이터 드리븐 및 BGM 전환 정상
- 1st_Road_to_Stage1부터 Stage2까지 흐름 안정적

다음 목표:
- Stage2Group NPC 상호작용 및 퀘스트 완료 => Stage2 마무리
- Stage1-2 호박 획득 및 요리 연계
- CodexGroup 실제 콘텐츠 채우기
- Stage3Group부터 본격 작업
- HUD/인벤토리 데이터 드리븐 강화
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/OO_Character.xlsx
+++ b/JsonConverter/ExcelFiles/OO_Character.xlsx
@@ -122,10 +122,6 @@
   </si>
   <si>
     <t xml:space="preserve">Stage2 보스 </t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>character_LeeMongRyong_01</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
@@ -270,6 +266,10 @@
       </rPr>
       <t>.</t>
     </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>character_LeeMongRyong_01</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -902,16 +902,16 @@
     </row>
     <row r="11" spans="1:15" ht="15.75" customHeight="1">
       <c r="A11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>37</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>

</xml_diff>